<commit_message>
se hace archivo py sin warnings
</commit_message>
<xml_diff>
--- a/Valuaciones_USA/ADBE_razones_financieras.xlsx
+++ b/Valuaciones_USA/ADBE_razones_financieras.xlsx
@@ -1686,105 +1686,65 @@
 *Menor a 4 indica baja rotación</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="V17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U17" t="n">
+        <v>0</v>
+      </c>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18">

</xml_diff>